<commit_message>
fix: rename equipment labels and clear old reason on reserve
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-50_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-50_Test_Cases.xlsx
@@ -597,7 +597,7 @@
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>Reserved and Partially fulfilled cannot be chosen by hand, and a reserved line can only become Unavailable</t>
+          <t>Reserved and Partially fulfilled cannot be chosen by hand, and a reserved line can only become 'Cannot be provided'</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>Line marked Unavailable can be reopened to Under review</t>
+          <t>Line marked 'Cannot be provided' can be reopened to Under review</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Marking an item Unavailable without a real reason is blocked</t>
+          <t>Marking an item 'Cannot be provided' without a real reason is blocked</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
@@ -725,7 +725,7 @@
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>Marking a reserved line Unavailable releases its reserved units</t>
+          <t>Marking a reserved line 'Cannot be provided' releases its units, and reserving it again clears the old reason</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
@@ -1407,7 +1407,7 @@
         <is>
           <t>1. Open the equipment request for the Robotics Expo event
 2. On the Confidence Monitor line, click 'Update'
-3. In 'Fulfilment status', choose 'Unavailable'
+3. In 'Fulfilment status', choose 'Cannot be provided'
 4. Paste the 501-character test text into 'Technical notes'
 5. Click 'Save'
 6. Delete one character, leaving 500
@@ -1437,7 +1437,7 @@
       <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Step 5: The error 'Technical notes must be 500 characters or fewer.' is shown under Technical notes. The Status chip still shows 'Requested' and nothing is saved.
-Step 7: 'Update saved.' appears and the Status chip shows 'Unavailable'.
+Step 7: 'Update saved.' appears and the Status chip shows 'Cannot be provided'.
 Step 8: All 500 characters are shown in the line's technical notes; nothing is cut off.</t>
         </is>
       </c>
@@ -1559,7 +1559,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Run TC05 first: Robotics Expo's Confidence Monitor is 'Unavailable' with a reason.
+          <t>Run TC05 first: Robotics Expo's Confidence Monitor is 'Cannot be provided' with a reason.
 Logged in as the assigned Coordinator, daniel.tan@connectsphere.com (password123).</t>
         </is>
       </c>
@@ -1599,7 +1599,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 4: Confidence Monitor shows the status chip 'Unavailable' and 'Technical Support notes: Only 1 working unit; suggest 2x 55-inch TV on stands as an alternative'. The notes are read-only for the Coordinator; their own Quantity and Technical requirements fields are still editable.</t>
+          <t>Step 4: Confidence Monitor shows the status chip 'Cannot be provided' and 'Technical Support notes: Only 1 working unit; suggest 2x 55-inch TV on stands as an alternative'. The notes are read-only for the Coordinator; their own Quantity and Technical requirements fields are still editable.</t>
         </is>
       </c>
     </row>
@@ -1720,7 +1720,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Run TC05 first: Robotics Expo's Confidence Monitor is 'Unavailable' with a reason.
+          <t>Run TC05 first: Robotics Expo's Confidence Monitor is 'Cannot be provided' with a reason.
 Event 'Design Week' also requests 'Confidence Monitor' x1, status 'Requested', no notes.
 Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).</t>
         </is>
@@ -1752,7 +1752,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="44.5" customHeight="1">
+    <row r="6" ht="58" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1760,7 +1760,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 3: Design Week's Confidence Monitor line still shows 'Requested' with no Technical Support notes. The 'Unavailable' status and reason from Robotics Expo do not appear here.</t>
+          <t>Step 3: Design Week's Confidence Monitor line still shows 'Requested' with no Technical Support notes. The 'Cannot be provided' status and reason from Robotics Expo do not appear here.</t>
         </is>
       </c>
     </row>
@@ -2333,7 +2333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2369,24 +2369,24 @@
       </c>
       <c r="C2" s="11" t="n"/>
     </row>
-    <row r="3" ht="71.5" customHeight="1">
+    <row r="3" ht="85" customHeight="1">
       <c r="A3" s="11" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="11" t="inlineStr">
         <is>
-          <t>OPEN - Reserve button on an Unavailable line: with the current SPM-49 code (canOfferReserve), an Unavailable line still offers Reserve once stock frees up. Both options are consistent. Allowing it is more convenient; requiring a reopen to 'Under review' first (TC04) is more deliberate. Product call, so no case is written until it is decided.</t>
+          <t>DECIDED (Janelle, 2 Oct) - Reserve stays on a line marked 'Cannot be provided': if stock frees up, Technical Support can reserve it in one click. Reserving it clears the old 'cannot be provided' reason, so the line never shows 'Reserved' next to a reason that no longer holds (TC07; reserveClearsStaffNotes() in src/lib/equipmentFulfilment.ts, used by the SPM-49 reserve route).</t>
         </is>
       </c>
       <c r="C3" s="11" t="n"/>
     </row>
-    <row r="4" ht="71.5" customHeight="1">
+    <row r="4" ht="58" customHeight="1">
       <c r="A4" s="11" t="n">
         <v>3</v>
       </c>
       <c r="B4" s="11" t="inlineStr">
         <is>
-          <t>OPEN - getting from the Equipment request page to the event: Technical Support has no Events item in the side menu, and the Equipment request page has no link to the event. The page now shows the Coordinator's technical requirements, so Technical Support may never need to leave it, and no test case depends on the link. Team to confirm.</t>
+          <t>DECIDED (Janelle, 2 Oct) - no link from the Equipment request page back to the event. The page shows everything Technical Support needs (the Coordinator's requirements, status, notes), and no test case depends on the link.</t>
         </is>
       </c>
       <c r="C4" s="11" t="n"/>
@@ -2402,13 +2402,13 @@
       </c>
       <c r="C5" s="11" t="n"/>
     </row>
-    <row r="6" ht="112" customHeight="1">
+    <row r="6" ht="166" customHeight="1">
       <c r="A6" s="11" t="n">
         <v>5</v>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>OPEN - fulfilment status vs approve/reject (Kristen's comment on the ticket): venue booking has request then approve/reject (SPM-42 then SPM-43), but equipment goes record, check, reserve (SPM-47, 48, 49) with fulfilment statuses. Every story in the SPM-47 to SPM-50 chain is written against the fulfilment-status model, so switching would mean revisiting ACs on shipped stories. Team to confirm the divergence is intentional; meanwhile these cases follow the model already used across the chain.</t>
+          <t>OPEN (answered by customer Q&amp;A #19) - fulfilment status vs approve/reject (Kristen's comment on the ticket): venue booking has request then approve/reject (SPM-42 then SPM-43), but equipment goes record, check, reserve (SPM-47, 48, 49) with fulfilment statuses. Every story in the SPM-47 to SPM-50 chain is written against the fulfilment-status model, so switching would mean revisiting ACs on shipped stories. Team to confirm the divergence is intentional; meanwhile these cases follow the model already used across the chain. Customer Q&amp;A #19 asked whether equipment has a formal request → approval workflow like venue booking: the answer is that the Coordinator records the requirement, Technical Support reviews suitability and availability, and available equipment can then be reserved - no approval step.</t>
         </is>
       </c>
       <c r="C6" s="11" t="n"/>
@@ -2435,57 +2435,57 @@
       </c>
       <c r="C8" s="11" t="n"/>
     </row>
-    <row r="9" ht="85" customHeight="1">
+    <row r="9" ht="98.5" customHeight="1">
       <c r="A9" s="11" t="n">
         <v>8</v>
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>DECIDED - hand-pickable statuses (TC02, TC03): 'Reserved' and 'Partially fulfilled' are set only by the Reserve button, which keeps Reserved = the smaller of requested and available everywhere (the SPM-49 rule). 'Requested' can be chosen to undo 'Under review'. A Reserved or Partially fulfilled line cannot be moved back to 'Requested' or 'Under review'; leaving it goes through 'Unavailable' with a reason.</t>
+          <t>DECIDED (Janelle, 2 Oct) - labels: the request status 'unavailable' is shown as 'Cannot be provided' (Technical Support's decision) and the availability result 'unavailable' as 'None available' (no stock free for those dates), so the two never read the same on one line. Only the displayed text changed; the stored value is still 'unavailable'. Differs from the S-25 mockup, which says 'Unavailable'. SPM-48/49 expected results updated to match.</t>
         </is>
       </c>
       <c r="C9" s="11" t="n"/>
     </row>
-    <row r="10" ht="44.5" customHeight="1">
+    <row r="10" ht="85" customHeight="1">
       <c r="A10" s="11" t="n">
         <v>9</v>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>DECIDED - reason for Unavailable (TC06, TC09): required, as Q&amp;A #90 needs text the Coordinator can act on. Technical notes are capped at 500 characters to match SPM-55's out-of-service reason.</t>
+          <t>DECIDED - hand-pickable statuses (TC02, TC03): 'Reserved' and 'Partially fulfilled' are set only by the Reserve button, which keeps Reserved = the smaller of requested and available everywhere (the SPM-49 rule). 'Requested' can be chosen to undo 'Under review'. A Reserved or Partially fulfilled line cannot be moved back to 'Requested' or 'Under review'; leaving it goes through 'Cannot be provided' with a reason.</t>
         </is>
       </c>
       <c r="C10" s="11" t="n"/>
     </row>
-    <row r="11" ht="112" customHeight="1">
+    <row r="11" ht="44.5" customHeight="1">
       <c r="A11" s="11" t="n">
         <v>10</v>
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>DECIDED - releasing stock when a line is marked Unavailable (TC07): availability counts only lines with status 'reserved' or 'partially_fulfilled' (committedQuantity in src/lib/equipmentAvailability.ts), so the status change alone frees the units, whatever is left in quantityReserved. TC07 therefore checks the other event's availability, not the stored field. Clearing quantityReserved when marking Unavailable is still recommended as data hygiene, so no row reads 'unavailable' with 1 reserved, but it is not needed for correctness.</t>
+          <t>DECIDED - reason for 'Cannot be provided' (TC06, TC09): required, as Q&amp;A #90 needs text the Coordinator can act on. Technical notes are capped at 500 characters to match SPM-55's out-of-service reason.</t>
         </is>
       </c>
       <c r="C11" s="11" t="n"/>
     </row>
-    <row r="12" ht="58" customHeight="1">
+    <row r="12" ht="112" customHeight="1">
       <c r="A12" s="11" t="n">
         <v>11</v>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>DECIDED - technical notes storage (TC08, TC10): stored in the existing EquipmentRequest.staffNotes column, separate from the Coordinator's technicalRequirements. The assigned Coordinator and the owning Organiser see them read-only.</t>
+          <t>DECIDED - releasing stock when a line is marked 'Cannot be provided' (TC07): availability counts only lines with status 'reserved' or 'partially_fulfilled' (committedQuantity in src/lib/equipmentAvailability.ts), so the status change alone frees the units, whatever is left in quantityReserved. TC07 therefore checks the other event's availability, not the stored field. Clearing quantityReserved when marking 'Cannot be provided' is still recommended as data hygiene, so no row reads 'unavailable' with 1 reserved, but it is not needed for correctness.</t>
         </is>
       </c>
       <c r="C12" s="11" t="n"/>
     </row>
-    <row r="13" ht="44.5" customHeight="1">
+    <row r="13" ht="58" customHeight="1">
       <c r="A13" s="11" t="n">
         <v>12</v>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>ANSWERED, out of scope - notifying the Coordinator when an item is marked Unavailable belongs to the batched notification story, so no case is written here (same position as SPM-49).</t>
+          <t>DECIDED - technical notes storage (TC08, TC10): stored in the existing EquipmentRequest.staffNotes column, separate from the Coordinator's technicalRequirements. The assigned Coordinator and the owning Organiser see them read-only.</t>
         </is>
       </c>
       <c r="C13" s="11" t="n"/>
@@ -2496,21 +2496,32 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>BUILT (AC1) - the Equipment request page now shows each line's 'Technical requirements' from the Coordinator, 'Technical Support notes', and 'Last updated by' (TC01, TC08, TC08).</t>
+          <t>ANSWERED, out of scope - notifying the Coordinator when an item is marked 'Cannot be provided' belongs to the batched notification story, so no case is written here (same position as SPM-49).</t>
         </is>
       </c>
       <c r="C14" s="11" t="n"/>
     </row>
-    <row r="15" ht="85" customHeight="1">
+    <row r="15" ht="44.5" customHeight="1">
       <c r="A15" s="11" t="n">
         <v>14</v>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
+          <t>BUILT (AC1) - the Equipment request page now shows each line's 'Technical requirements' from the Coordinator, 'Technical Support notes', and 'Last updated by' (TC01, TC08, TC08).</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="n"/>
+    </row>
+    <row r="16" ht="85" customHeight="1">
+      <c r="A16" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
           <t>Test data - `npm run fixtures:spm50` (scripts/seed-spm50.ts) creates or resets the SPM-50 events: Robotics Expo, Design Week, Charity Briefing, Charity Gala, Cancelled Hackathon and Pending Showcase (Aug-Sep 2027, assigned Coordinator daniel.tan, Robotics Expo owned by Rachel Ng). prisma/seed.ts creates the same rows. Run the script again before repeating any case that saves a change.</t>
         </is>
       </c>
-      <c r="C15" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2898,7 +2909,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Rule (team decision): 'Reserved' and 'Partially fulfilled' mean stock is held, so only the Reserve button (SPM-49), which checks availability, can set them. Leaving them releases stock, so a reserved line can only be marked 'Unavailable' (with a reason, TC07).
+          <t>Rule (team decision): 'Reserved' and 'Partially fulfilled' mean stock is held, so only the Reserve button (SPM-49), which checks availability, can set them. Leaving them releases stock, so a reserved line can only be marked 'Cannot be provided' (with a reason, TC07).
 Robotics Expo's Wireless Presenter line is 'Requested'. Charity Briefing's Mobile Charging Cart line is 'Reserved' (Reserved = 1).
 Data: run `npm run fixtures:spm50` first.
 Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).</t>
@@ -2943,8 +2954,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 3: The list offers 'Requested', 'Under review' and 'Unavailable' only. 'Reserved' and 'Partially fulfilled' are not offered. The Reserve button remains on the line.
-Step 7: The list offers 'Reserved' (the current status) and 'Unavailable' only. 'Requested' and 'Under review' are not offered.</t>
+          <t>Step 3: The list offers 'Requested', 'Under review' and 'Cannot be provided' only. 'Reserved' and 'Partially fulfilled' are not offered. The Reserve button remains on the line.
+Step 7: The list offers 'Reserved' (the current status) and 'Cannot be provided' only. 'Requested' and 'Under review' are not offered.</t>
         </is>
       </c>
     </row>
@@ -3065,7 +3076,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Event 'Design Week' (2027-08-16, status 'Planning') has a 'Ring Light' x2 line already marked 'Unavailable' with technical notes 'Both units out for repair'.
+          <t>Event 'Design Week' (2027-08-16, status 'Planning') has a 'Ring Light' x2 line already marked 'Cannot be provided' with technical notes 'Both units out for repair'.
 Data: run `npm run fixtures:spm50` first, and again before repeating the case.
 Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).</t>
         </is>
@@ -3095,7 +3106,7 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Fulfilment status: Unavailable -&gt; Under review
+          <t>Fulfilment status: Cannot be provided -&gt; Under review
 Technical notes: Repair finished early, re-checking availability</t>
         </is>
       </c>
@@ -3245,7 +3256,7 @@
         <is>
           <t>1. Open the equipment request for the Robotics Expo event
 2. On the Confidence Monitor line, click 'Update'
-3. In 'Fulfilment status', choose 'Unavailable'
+3. In 'Fulfilment status', choose 'Cannot be provided'
 4. In 'Technical notes', enter the test data
 5. Click 'Save'
 6. Refresh the page
@@ -3261,7 +3272,7 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Fulfilment status: Unavailable
+          <t>Fulfilment status: Cannot be provided
 Technical notes: Only 1 working unit; suggest 2x 55-inch TV on stands as an alternative</t>
         </is>
       </c>
@@ -3274,8 +3285,8 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 5: 'Update saved.' appears. The Status chip shows 'Unavailable' (red).
-Step 6: The Status chip still shows 'Unavailable' and the notes 'Only 1 working unit; suggest 2x 55-inch TV on stands as an alternative' are shown on the line after 'Technical Support notes:'.
+          <t>Step 5: 'Update saved.' appears. The Status chip shows 'Cannot be provided' (red).
+Step 6: The Status chip still shows 'Cannot be provided' and the notes 'Only 1 working unit; suggest 2x 55-inch TV on stands as an alternative' are shown on the line after 'Technical Support notes:'.
 Step 7: The Wireless Presenter line still shows the Status chip 'Requested' and no Technical Support notes. Because the lines are no longer at the same stage, the 'Requested items' header shows no single status chip.</t>
         </is>
       </c>
@@ -3413,7 +3424,7 @@
         <is>
           <t>1. Open the equipment request for the Robotics Expo event
 2. On the Confidence Monitor line, click 'Update'
-3. In 'Fulfilment status', choose 'Unavailable'
+3. In 'Fulfilment status', choose 'Cannot be provided'
 4. Leave 'Technical notes' empty
 5. Click 'Save'
 6. In 'Technical notes', type three spaces
@@ -3429,7 +3440,7 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Fulfilment status: Unavailable
+          <t>Fulfilment status: Cannot be provided
 Technical notes: (empty), then '   ' (3 spaces)</t>
         </is>
       </c>
@@ -3564,7 +3575,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Rule: only lines with status 'Reserved' or 'Partially fulfilled' count against stock, so changing the status to 'Unavailable' frees the units by itself.
+          <t>Rule: only lines with status 'Reserved' or 'Partially fulfilled' count against stock, so changing the status to 'Cannot be provided' frees the units by itself.
 'Mobile Charging Cart' has 1 unit in total.
 Event 'Charity Briefing' (2027-08-23) has 1x Mobile Charging Cart already 'Reserved' (Reserved = 1).
 Event 'Charity Gala' (same date, overlapping times) requests 1x Mobile Charging Cart, status 'Requested'.
@@ -3573,7 +3584,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="125.5" customHeight="1">
+    <row r="4" ht="152.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -3585,10 +3596,12 @@
 2. Read the Mobile Charging Cart line
 3. Click Equipment Requests in the breadcrumb and open the Charity Briefing event
 4. On the Mobile Charging Cart line, click 'Update'
-5. In 'Fulfilment status', choose 'Unavailable'
+5. In 'Fulfilment status', choose 'Cannot be provided'
 6. In 'Technical notes', enter the test data
 7. Click 'Save'
-8. Go back to the Charity Gala equipment request</t>
+8. Go back to the Charity Gala equipment request
+9. Go back to the Charity Briefing equipment request
+10. Click Reserve on the Mobile Charging Cart line</t>
         </is>
       </c>
     </row>
@@ -3605,7 +3618,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="139" customHeight="1">
+    <row r="6" ht="206.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -3613,9 +3626,10 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 2: Charity Gala's line shows '1 total − 0 in maintenance − 1 reserved elsewhere = 0 available' and the Availability chip 'Unavailable', with 'Held by Charity Briefing (1 unit)'.
-Step 7: Charity Briefing's line shows the Status chip 'Unavailable'.
-Step 8: Charity Gala's line now shows '1 total − 0 in maintenance − 0 reserved elsewhere = 1 available' with the Availability chip 'Available'. Charity Briefing is no longer listed as holding it, and the Reserve button is offered.</t>
+          <t>Step 2: Charity Gala's line shows '1 total − 0 in maintenance − 1 reserved elsewhere = 0 available' and the Availability chip 'None available', with 'Held by Charity Briefing (1 unit)'.
+Step 7: Charity Briefing's line shows the Status chip 'Cannot be provided'.
+Step 8: Charity Gala's line now shows '1 total − 0 in maintenance − 0 reserved elsewhere = 1 available' with the Availability chip 'Available'. Charity Briefing is no longer listed as holding it, and the Reserve button is offered.
+Step 10: 'Reservation saved: 1 reserved.' appears. The Status chip shows 'Reserved', the Reserved box shows 1, and the line shows 'Technical Support notes: —': the old reason 'Cart battery failed inspection, cannot be sent out' is cleared, because it no longer holds.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: Technical Support sees equipment from Planning only
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-50_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-50_Test_Cases.xlsx
@@ -917,12 +917,12 @@
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Lines on a cancelled event cannot be updated</t>
+          <t>A confirmed event's equipment is shown but cannot be changed</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>AC2, AC3, AC4</t>
+          <t>AC1, AC2, AC3, AC4</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
@@ -932,7 +932,7 @@
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Acceptance Criteria</t>
         </is>
       </c>
     </row>
@@ -949,12 +949,12 @@
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>Equipment on an event that is not yet approved cannot be updated</t>
+          <t>Technical Support does not see an event's equipment before the Coordinator starts planning</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>AC2, AC3, AC4</t>
+          <t>AC1, AC2</t>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr">
@@ -988,7 +988,7 @@
       </c>
       <c r="F20" s="9" t="n"/>
     </row>
-    <row r="21" ht="17.5" customHeight="1">
+    <row r="21" ht="44.5" customHeight="1">
       <c r="A21" s="11" t="inlineStr">
         <is>
           <t>AC1</t>
@@ -1003,7 +1003,9 @@
       <c r="D21" s="9" t="n"/>
       <c r="E21" s="11" t="inlineStr">
         <is>
-          <t>SPM-50-TC01</t>
+          <t>SPM-50-TC01
+SPM-50-TC13
+SPM-50-TC14</t>
         </is>
       </c>
       <c r="F21" s="9" t="n"/>
@@ -1034,7 +1036,7 @@
       </c>
       <c r="F22" s="9" t="n"/>
     </row>
-    <row r="23" ht="98.5" customHeight="1">
+    <row r="23" ht="85" customHeight="1">
       <c r="A23" s="11" t="inlineStr">
         <is>
           <t>AC3</t>
@@ -1054,13 +1056,12 @@
 SPM-50-TC06
 SPM-50-TC07
 SPM-50-TC09
-SPM-50-TC13
-SPM-50-TC14</t>
+SPM-50-TC13</t>
         </is>
       </c>
       <c r="F23" s="9" t="n"/>
     </row>
-    <row r="24" ht="71.5" customHeight="1">
+    <row r="24" ht="58" customHeight="1">
       <c r="A24" s="11" t="inlineStr">
         <is>
           <t>AC4</t>
@@ -1078,8 +1079,7 @@
           <t>SPM-50-TC08
 SPM-50-TC09
 SPM-50-TC12
-SPM-50-TC13
-SPM-50-TC14</t>
+SPM-50-TC13</t>
         </is>
       </c>
       <c r="F24" s="9" t="n"/>
@@ -2035,7 +2035,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="58" customHeight="1">
+    <row r="3" ht="139" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2043,12 +2043,14 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Event 'Cancelled Hackathon' (2027-08-30, status 'Cancelled') requests 2x Wireless Presenter, status 'Requested'.
+          <t>Rule (team decision, 3 Oct, following the BPMN): Technical Support checks, reserves and updates equipment while the event is in Planning. Once the event is Confirmed its equipment is final - they still see it, to prepare it, but a change goes through a change request.
+Event 'Confirmed Launch' (2027-08-30, status 'Confirmed') has 2x Wireless Presenter, status 'Reserved' (Reserved = 2).
+Data: run `npm run fixtures:spm50` first.
 Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="71.5" customHeight="1">
+    <row r="4" ht="58" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2057,8 +2059,8 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the Cancelled Hackathon event
-3. Look for an 'Update' button on the Wireless Presenter line</t>
+2. Open the equipment request for the Confirmed Launch event
+3. Look for an 'Update' or 'Reserve' button on the Wireless Presenter line</t>
         </is>
       </c>
     </row>
@@ -2070,11 +2072,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Event status: Cancelled</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="85" customHeight="1">
+          <t>Event status: Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="112" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2082,9 +2084,9 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 1: Cancelled Hackathon is listed with Event status 'Cancelled'.
-Step 2: The page shows 'This event is cancelled — equipment can no longer be reserved.'
-Step 3: No 'Update' button and no Reserve button are shown. The line still shows 'Requested' with Requested 2.</t>
+          <t>Step 1: Confirmed Launch is listed, with Event status 'Confirmed'.
+Step 2: The page shows 'This event is confirmed — its equipment is final. A change now goes through a change request.' The Wireless Presenter line shows the Status chip 'Reserved' and Reserved 2.
+Step 3: No 'Update' button and no 'Reserve' button are shown.</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2199,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="112" customHeight="1">
+    <row r="3" ht="179.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2205,14 +2207,15 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Rule (team decision, 2 Oct): until Operations approves an event, only its Organiser and Coordinator work on it. Technical Support starts once it is Approved.
-Event 'Pending Showcase' (2027-09-06, status 'Under review') requests 1x Wireless Presenter, status 'Requested'.
+          <t>Rule (team decision, 3 Oct, following the BPMN): Technical Support's lane starts after the Coordinator's 'Record equipment request' - in Planning. Before that, the equipment is only part of the organiser's request.
+Event 'Pending Showcase' (2027-09-06, status 'Under review') and event 'Approved Briefing' (2027-09-13, status 'Approved', the Coordinator has not started planning) each request 1x Wireless Presenter.
+Their references (EVT-…) are printed by `npm run fixtures:spm50`.
 Data: run `npm run fixtures:spm50` first.
 Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="58" customHeight="1">
+    <row r="4" ht="98.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2221,8 +2224,9 @@
       <c r="B4" s="13" t="inlineStr">
         <is>
           <t>1. Click Equipment Requests in the side menu
-2. Open the equipment request for the Pending Showcase event
-3. Look for an 'Update' button on the Wireless Presenter line</t>
+2. Look for Pending Showcase and Approved Briefing in the list
+3. Type /equipment/requests/&lt;Pending Showcase's reference&gt; into the address bar
+4. Type /equipment/requests/&lt;Approved Briefing's reference&gt; into the address bar</t>
         </is>
       </c>
     </row>
@@ -2234,11 +2238,11 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Event status: Under review</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
+          <t>Event statuses: Under review, Approved</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="71.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2246,8 +2250,9 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Step 2: The page shows 'This event is under review — equipment requests can be updated once the event is approved.'
-Step 3: No 'Update' button is shown. The line still shows 'Requested' with Requested 1.</t>
+          <t>Step 2: Neither event is listed.
+Step 3: The page shows 'This event was not found, or its equipment is not ready for Technical Support yet.' No equipment lines, Update or Reserve buttons are shown.
+Step 4: The same message is shown for Approved Briefing.</t>
         </is>
       </c>
     </row>
@@ -2333,7 +2338,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2413,79 +2418,79 @@
       </c>
       <c r="C6" s="11" t="n"/>
     </row>
-    <row r="7" ht="98.5" customHeight="1">
+    <row r="7" ht="166" customHeight="1">
       <c r="A7" s="11" t="n">
         <v>6</v>
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>IN PROGRESS (Kristen, her status story) - SPM-49's Reserve button is not limited the same way yet: it still works on Submitted and Under review events (eventAllowsReserving in src/lib/equipmentAvailability.ts). Until Kristen's change lands, Pending Showcase (TC14) still offers Reserve while Update is not offered. TC14 checks only the Update button. Her change also needs SPM-49's seeded events moved from 'Under review' to 'Planning'.</t>
+          <t>DECIDED (Kristen, 3 Oct, following the BPMN) - Technical Support sees an event's equipment only in Planning and Confirmed (TECH_SUPPORT_EQUIPMENT_STATUSES): the BPMN's Technical Support lane starts after the Coordinator's 'Record equipment request', with 'Check equipment availability' and 'Reserve equipment' in Planning and 'Prepare equipment' in Confirmed. Checking, reserving and updating happen in Planning only; Confirmed is read-only (TC13). Before Planning - including Approved, when the Coordinator has not started - and after it (postponed, cancelled, rejected, completed) the event is not listed and a direct link says it is not found (TC14). Not in SPM-48/49/50's ACs: a process alignment, applied to all three; supersedes the earlier 'Approved onwards' rule and the Reserve gap.</t>
         </is>
       </c>
       <c r="C7" s="11" t="n"/>
     </row>
-    <row r="8" ht="85" customHeight="1">
+    <row r="8" ht="98.5" customHeight="1">
       <c r="A8" s="11" t="n">
         <v>7</v>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>DECIDED (Kristen, 2 Oct) - Technical Support only updates an event's equipment once the event is Approved, Planning or Confirmed (TC14). Before approval only the Organiser and Coordinator work on it, as there is no point arranging equipment for an event that may be rejected. Completed, cancelled, rejected and postponed events cannot be updated either (TC13).</t>
+          <t>DECIDED (Janelle, 2 Oct) - labels: the request status 'unavailable' is shown as 'Cannot be provided' (Technical Support's decision) and the availability result 'unavailable' as 'None available' (no stock free for those dates), so the two never read the same on one line. Only the displayed text changed; the stored value is still 'unavailable'. Differs from the S-25 mockup, which says 'Unavailable'. SPM-48/49 expected results updated to match.</t>
         </is>
       </c>
       <c r="C8" s="11" t="n"/>
     </row>
-    <row r="9" ht="98.5" customHeight="1">
+    <row r="9" ht="85" customHeight="1">
       <c r="A9" s="11" t="n">
         <v>8</v>
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>DECIDED (Janelle, 2 Oct) - labels: the request status 'unavailable' is shown as 'Cannot be provided' (Technical Support's decision) and the availability result 'unavailable' as 'None available' (no stock free for those dates), so the two never read the same on one line. Only the displayed text changed; the stored value is still 'unavailable'. Differs from the S-25 mockup, which says 'Unavailable'. SPM-48/49 expected results updated to match.</t>
+          <t>DECIDED - hand-pickable statuses (TC02, TC03): 'Reserved' and 'Partially fulfilled' are set only by the Reserve button, which keeps Reserved = the smaller of requested and available everywhere (the SPM-49 rule). 'Requested' can be chosen to undo 'Under review'. A Reserved or Partially fulfilled line cannot be moved back to 'Requested' or 'Under review'; leaving it goes through 'Cannot be provided' with a reason.</t>
         </is>
       </c>
       <c r="C9" s="11" t="n"/>
     </row>
-    <row r="10" ht="85" customHeight="1">
+    <row r="10" ht="44.5" customHeight="1">
       <c r="A10" s="11" t="n">
         <v>9</v>
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>DECIDED - hand-pickable statuses (TC02, TC03): 'Reserved' and 'Partially fulfilled' are set only by the Reserve button, which keeps Reserved = the smaller of requested and available everywhere (the SPM-49 rule). 'Requested' can be chosen to undo 'Under review'. A Reserved or Partially fulfilled line cannot be moved back to 'Requested' or 'Under review'; leaving it goes through 'Cannot be provided' with a reason.</t>
+          <t>DECIDED - reason for 'Cannot be provided' (TC06, TC09): required, as Q&amp;A #90 needs text the Coordinator can act on. Technical notes are capped at 500 characters to match SPM-55's out-of-service reason.</t>
         </is>
       </c>
       <c r="C10" s="11" t="n"/>
     </row>
-    <row r="11" ht="44.5" customHeight="1">
+    <row r="11" ht="112" customHeight="1">
       <c r="A11" s="11" t="n">
         <v>10</v>
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>DECIDED - reason for 'Cannot be provided' (TC06, TC09): required, as Q&amp;A #90 needs text the Coordinator can act on. Technical notes are capped at 500 characters to match SPM-55's out-of-service reason.</t>
+          <t>DECIDED - releasing stock when a line is marked 'Cannot be provided' (TC07): availability counts only lines with status 'reserved' or 'partially_fulfilled' (committedQuantity in src/lib/equipmentAvailability.ts), so the status change alone frees the units, whatever is left in quantityReserved. TC07 therefore checks the other event's availability, not the stored field. Clearing quantityReserved when marking 'Cannot be provided' is still recommended as data hygiene, so no row reads 'unavailable' with 1 reserved, but it is not needed for correctness.</t>
         </is>
       </c>
       <c r="C11" s="11" t="n"/>
     </row>
-    <row r="12" ht="112" customHeight="1">
+    <row r="12" ht="58" customHeight="1">
       <c r="A12" s="11" t="n">
         <v>11</v>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>DECIDED - releasing stock when a line is marked 'Cannot be provided' (TC07): availability counts only lines with status 'reserved' or 'partially_fulfilled' (committedQuantity in src/lib/equipmentAvailability.ts), so the status change alone frees the units, whatever is left in quantityReserved. TC07 therefore checks the other event's availability, not the stored field. Clearing quantityReserved when marking 'Cannot be provided' is still recommended as data hygiene, so no row reads 'unavailable' with 1 reserved, but it is not needed for correctness.</t>
+          <t>DECIDED - technical notes storage (TC08, TC10): stored in the existing EquipmentRequest.staffNotes column, separate from the Coordinator's technicalRequirements. The assigned Coordinator and the owning Organiser see them read-only.</t>
         </is>
       </c>
       <c r="C12" s="11" t="n"/>
     </row>
-    <row r="13" ht="58" customHeight="1">
+    <row r="13" ht="44.5" customHeight="1">
       <c r="A13" s="11" t="n">
         <v>12</v>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>DECIDED - technical notes storage (TC08, TC10): stored in the existing EquipmentRequest.staffNotes column, separate from the Coordinator's technicalRequirements. The assigned Coordinator and the owning Organiser see them read-only.</t>
+          <t>ANSWERED, out of scope - notifying the Coordinator when an item is marked 'Cannot be provided' belongs to the batched notification story, so no case is written here (same position as SPM-49).</t>
         </is>
       </c>
       <c r="C13" s="11" t="n"/>
@@ -2496,32 +2501,21 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>ANSWERED, out of scope - notifying the Coordinator when an item is marked 'Cannot be provided' belongs to the batched notification story, so no case is written here (same position as SPM-49).</t>
+          <t>BUILT (AC1) - the Equipment request page now shows each line's 'Technical requirements' from the Coordinator, 'Technical Support notes', and 'Last updated by' (TC01, TC08, TC08).</t>
         </is>
       </c>
       <c r="C14" s="11" t="n"/>
     </row>
-    <row r="15" ht="44.5" customHeight="1">
+    <row r="15" ht="85" customHeight="1">
       <c r="A15" s="11" t="n">
         <v>14</v>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>BUILT (AC1) - the Equipment request page now shows each line's 'Technical requirements' from the Coordinator, 'Technical Support notes', and 'Last updated by' (TC01, TC08, TC08).</t>
+          <t>Test data - `npm run fixtures:spm50` (scripts/seed-spm50.ts) creates or resets the SPM-50 events: Robotics Expo, Design Week, Charity Briefing, Charity Gala, Confirmed Launch, Pending Showcase and Approved Briefing (Aug-Sep 2027, assigned Coordinator daniel.tan, Robotics Expo owned by Rachel Ng). prisma/seed.ts creates the same rows. Run the script again before repeating any case that saves a change.</t>
         </is>
       </c>
       <c r="C15" s="11" t="n"/>
-    </row>
-    <row r="16" ht="85" customHeight="1">
-      <c r="A16" s="11" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="11" t="inlineStr">
-        <is>
-          <t>Test data - `npm run fixtures:spm50` (scripts/seed-spm50.ts) creates or resets the SPM-50 events: Robotics Expo, Design Week, Charity Briefing, Charity Gala, Cancelled Hackathon and Pending Showcase (Aug-Sep 2027, assigned Coordinator daniel.tan, Robotics Expo owned by Rachel Ng). prisma/seed.ts creates the same rows. Run the script again before repeating any case that saves a change.</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
SPM-102: Keep an equipment line's controls beside long technical notes
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-50_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-50_Test_Cases.xlsx
@@ -488,6 +488,7 @@
       <c r="E1" s="8" t="n"/>
       <c r="F1" s="9" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
@@ -968,6 +969,8 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
@@ -1106,6 +1109,7 @@
       </c>
       <c r="F25" s="9" t="n"/>
     </row>
+    <row r="26"/>
     <row r="27" ht="301" customHeight="1">
       <c r="A27" s="7" t="inlineStr">
         <is>
@@ -1268,7 +1272,7 @@
       <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Step 5: 'Update saved.' appears. The Status chip still shows 'Requested'.
-Step 6: The line shows 'Technical Support notes: Presenters need fresh AAA batteries; USB-C dongle is in kit bag 3', separately from 'Technical requirements: Must pair with the stage laptop over USB-C', which is unchanged. It also shows 'Last updated by Vikram Nair, ' followed by the date and time of the save (for example '2 Oct 2026, 14:05').
+Step 6: The line shows 'Technical Support notes: Presenters need fresh AAA batteries; USB-C dongle is in kit bag 3', separately from 'Technical requirements: Must pair with the stage laptop over USB-C', which is unchanged. It also shows 'Last updated by Vikram Nair, ' followed by the date and time of the save (for example '2 Oct 2026, 14:05'). The line's Requested, Reserved, Status and Availability boxes and its 'Update' and 'Reserve' buttons stay on the right of its details, level with the other lines, at any laptop window width - the long note wraps within the details (SPM-102).
 Step 9: 'Update saved.' appears and the line shows 'Technical Support notes: —'. The Status chip still shows 'Requested'.</t>
         </is>
       </c>

</xml_diff>